<commit_message>
完成 P2-04. P2-05 被阻塞。
</commit_message>
<xml_diff>
--- a/0_tasks.xlsx
+++ b/0_tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luessiaw\Nutstore\1\Thoughts\Others\20260514摄像头破解\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1ACEE59-C05F-47BE-ABCD-7BF9C79A4398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC3D628-A197-4CD2-931C-B370CD80781F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8910" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="317">
   <si>
     <t>P0-01</t>
   </si>
@@ -970,6 +970,9 @@
   </si>
   <si>
     <t>已完成</t>
+  </si>
+  <si>
+    <t>进行中</t>
   </si>
   <si>
     <t>测试常见 RTSP 地址</t>
@@ -1946,7 +1949,7 @@
         <v>16</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>71</v>
+        <v>313</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>113</v>
@@ -1962,13 +1965,13 @@
         <v>28</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>71</v>
+        <v>314</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>115</v>
@@ -2006,7 +2009,7 @@
         <v>30</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>26</v>

</xml_diff>